<commit_message>
Intro TU MV Cas S02b
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS S02/Cas S02.xlsx
+++ b/Manuel Validation/CAS S02/Cas S02.xlsx
@@ -527,7 +527,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -962,7 +962,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -974,7 +974,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -2196,8 +2196,8 @@
         <v>86</v>
       </c>
       <c r="E56" s="61">
-        <f>hw*tw*FyW/SQRT(3)/GammaM0/1000</f>
-        <v>1873.9140165697568</v>
+        <f>hw*tw*FyW/SQRT(3)/GammaM0/1000*Eta</f>
+        <v>2248.696819883708</v>
       </c>
       <c r="F56" t="s">
         <v>13</v>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="E58" s="60">
         <f>VEd_U1/VRd</f>
-        <v>0.19979571991533951</v>
+        <v>0.16649643326278291</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>26</v>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="E59" s="60">
         <f>VEd_U2/VRd</f>
-        <v>0.16329457877696019</v>
+        <v>0.13607881564746682</v>
       </c>
       <c r="M59" s="3"/>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="E60" s="75">
         <f>MAX(E58:E59)</f>
-        <v>0.19979571991533951</v>
+        <v>0.16649643326278291</v>
       </c>
       <c r="M60" s="3" t="s">
         <v>115</v>

</xml_diff>

<commit_message>
Correction bug label combi dans synthèse ELU
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS S02/Cas S02.xlsx
+++ b/Manuel Validation/CAS S02/Cas S02.xlsx
@@ -2622,6 +2622,10 @@
       <c r="F85" t="s">
         <v>7</v>
       </c>
+      <c r="G85">
+        <f>Fu</f>
+        <v>470</v>
+      </c>
       <c r="M85" s="3" t="s">
         <v>122</v>
       </c>

</xml_diff>